<commit_message>
fix(export): leva cada categoria para a coluna do Anexo I versao 19
O mapa de colunas era placeholder e mandava transporte e estacionamento
para W, que no formulario versao 19 e Combustivel: uma corrida de taxi
saia lancada como abastecimento. O template sintetico so tinha S, W e
X, e o total da linha era S+W+X (issue 38).

- Mapa da versao 19: Q para transporte, X para estacionamento,
  lavanderia e outros, W para combustivel, S para alimentacao.
- O template sintetico ganhou O, Q, S, U, W e X, com o total da linha
  cobrindo as seis; regenerado pelo script do projeto.
- Teste por categoria afirma a coluna e que ela entra no total da linha.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/anexo-i-template.xlsx
+++ b/assets/anexo-i-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>PRESTACAO DE CONTAS — ANEXO I (MODELO SINTETICO, NAO OFICIAL)</t>
   </si>
@@ -31,16 +31,25 @@
     <t>Descricao</t>
   </si>
   <si>
+    <t>Passagens</t>
+  </si>
+  <si>
+    <t>Taxi/Conducoes</t>
+  </si>
+  <si>
     <t>Alimentacao</t>
   </si>
   <si>
     <t>Pagamento</t>
   </si>
   <si>
-    <t>Transporte</t>
+    <t>Hospedagem</t>
   </si>
   <si>
-    <t>Hospedagem</t>
+    <t>Combustivel</t>
+  </si>
+  <si>
+    <t>Outras</t>
   </si>
   <si>
     <t>Total</t>
@@ -492,27 +501,45 @@
       <c r="G31" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="O31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q31" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="S31" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="U31" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="W31" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="X31" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Y31" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B32" s="3"/>
+      <c r="O32" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>0</v>
+      </c>
       <c r="S32" s="2">
         <v>0</v>
       </c>
+      <c r="U32" s="2">
+        <v>0</v>
+      </c>
       <c r="W32" s="2">
         <v>0</v>
       </c>
@@ -520,14 +547,23 @@
         <v>0</v>
       </c>
       <c r="Y32" s="2">
-        <f>S32+W32+X32</f>
+        <f>O32+Q32+S32+U32+W32+X32</f>
       </c>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B33" s="3"/>
+      <c r="O33" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>0</v>
+      </c>
       <c r="S33" s="2">
         <v>0</v>
       </c>
+      <c r="U33" s="2">
+        <v>0</v>
+      </c>
       <c r="W33" s="2">
         <v>0</v>
       </c>
@@ -535,14 +571,23 @@
         <v>0</v>
       </c>
       <c r="Y33" s="2">
-        <f>S33+W33+X33</f>
+        <f>O33+Q33+S33+U33+W33+X33</f>
       </c>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B34" s="3"/>
+      <c r="O34" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>0</v>
+      </c>
       <c r="S34" s="2">
         <v>0</v>
       </c>
+      <c r="U34" s="2">
+        <v>0</v>
+      </c>
       <c r="W34" s="2">
         <v>0</v>
       </c>
@@ -550,14 +595,23 @@
         <v>0</v>
       </c>
       <c r="Y34" s="2">
-        <f>S34+W34+X34</f>
+        <f>O34+Q34+S34+U34+W34+X34</f>
       </c>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B35" s="3"/>
+      <c r="O35" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>0</v>
+      </c>
       <c r="S35" s="2">
         <v>0</v>
       </c>
+      <c r="U35" s="2">
+        <v>0</v>
+      </c>
       <c r="W35" s="2">
         <v>0</v>
       </c>
@@ -565,14 +619,23 @@
         <v>0</v>
       </c>
       <c r="Y35" s="2">
-        <f>S35+W35+X35</f>
+        <f>O35+Q35+S35+U35+W35+X35</f>
       </c>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B36" s="3"/>
+      <c r="O36" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>0</v>
+      </c>
       <c r="S36" s="2">
         <v>0</v>
       </c>
+      <c r="U36" s="2">
+        <v>0</v>
+      </c>
       <c r="W36" s="2">
         <v>0</v>
       </c>
@@ -580,14 +643,23 @@
         <v>0</v>
       </c>
       <c r="Y36" s="2">
-        <f>S36+W36+X36</f>
+        <f>O36+Q36+S36+U36+W36+X36</f>
       </c>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B37" s="3"/>
+      <c r="O37" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>0</v>
+      </c>
       <c r="S37" s="2">
         <v>0</v>
       </c>
+      <c r="U37" s="2">
+        <v>0</v>
+      </c>
       <c r="W37" s="2">
         <v>0</v>
       </c>
@@ -595,14 +667,23 @@
         <v>0</v>
       </c>
       <c r="Y37" s="2">
-        <f>S37+W37+X37</f>
+        <f>O37+Q37+S37+U37+W37+X37</f>
       </c>
     </row>
     <row r="38" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B38" s="3"/>
+      <c r="O38" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>0</v>
+      </c>
       <c r="S38" s="2">
         <v>0</v>
       </c>
+      <c r="U38" s="2">
+        <v>0</v>
+      </c>
       <c r="W38" s="2">
         <v>0</v>
       </c>
@@ -610,14 +691,23 @@
         <v>0</v>
       </c>
       <c r="Y38" s="2">
-        <f>S38+W38+X38</f>
+        <f>O38+Q38+S38+U38+W38+X38</f>
       </c>
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B39" s="3"/>
+      <c r="O39" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>0</v>
+      </c>
       <c r="S39" s="2">
         <v>0</v>
       </c>
+      <c r="U39" s="2">
+        <v>0</v>
+      </c>
       <c r="W39" s="2">
         <v>0</v>
       </c>
@@ -625,14 +715,23 @@
         <v>0</v>
       </c>
       <c r="Y39" s="2">
-        <f>S39+W39+X39</f>
+        <f>O39+Q39+S39+U39+W39+X39</f>
       </c>
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B40" s="3"/>
+      <c r="O40" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>0</v>
+      </c>
       <c r="S40" s="2">
         <v>0</v>
       </c>
+      <c r="U40" s="2">
+        <v>0</v>
+      </c>
       <c r="W40" s="2">
         <v>0</v>
       </c>
@@ -640,14 +739,23 @@
         <v>0</v>
       </c>
       <c r="Y40" s="2">
-        <f>S40+W40+X40</f>
+        <f>O40+Q40+S40+U40+W40+X40</f>
       </c>
     </row>
     <row r="41" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B41" s="3"/>
+      <c r="O41" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>0</v>
+      </c>
       <c r="S41" s="2">
         <v>0</v>
       </c>
+      <c r="U41" s="2">
+        <v>0</v>
+      </c>
       <c r="W41" s="2">
         <v>0</v>
       </c>
@@ -655,14 +763,23 @@
         <v>0</v>
       </c>
       <c r="Y41" s="2">
-        <f>S41+W41+X41</f>
+        <f>O41+Q41+S41+U41+W41+X41</f>
       </c>
     </row>
     <row r="42" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B42" s="3"/>
+      <c r="O42" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>0</v>
+      </c>
       <c r="S42" s="2">
         <v>0</v>
       </c>
+      <c r="U42" s="2">
+        <v>0</v>
+      </c>
       <c r="W42" s="2">
         <v>0</v>
       </c>
@@ -670,14 +787,23 @@
         <v>0</v>
       </c>
       <c r="Y42" s="2">
-        <f>S42+W42+X42</f>
+        <f>O42+Q42+S42+U42+W42+X42</f>
       </c>
     </row>
     <row r="43" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B43" s="3"/>
+      <c r="O43" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="2">
+        <v>0</v>
+      </c>
       <c r="S43" s="2">
         <v>0</v>
       </c>
+      <c r="U43" s="2">
+        <v>0</v>
+      </c>
       <c r="W43" s="2">
         <v>0</v>
       </c>
@@ -685,14 +811,23 @@
         <v>0</v>
       </c>
       <c r="Y43" s="2">
-        <f>S43+W43+X43</f>
+        <f>O43+Q43+S43+U43+W43+X43</f>
       </c>
     </row>
     <row r="44" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B44" s="3"/>
+      <c r="O44" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="2">
+        <v>0</v>
+      </c>
       <c r="S44" s="2">
         <v>0</v>
       </c>
+      <c r="U44" s="2">
+        <v>0</v>
+      </c>
       <c r="W44" s="2">
         <v>0</v>
       </c>
@@ -700,14 +835,23 @@
         <v>0</v>
       </c>
       <c r="Y44" s="2">
-        <f>S44+W44+X44</f>
+        <f>O44+Q44+S44+U44+W44+X44</f>
       </c>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="3"/>
+      <c r="O45" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="2">
+        <v>0</v>
+      </c>
       <c r="S45" s="2">
         <v>0</v>
       </c>
+      <c r="U45" s="2">
+        <v>0</v>
+      </c>
       <c r="W45" s="2">
         <v>0</v>
       </c>
@@ -715,14 +859,23 @@
         <v>0</v>
       </c>
       <c r="Y45" s="2">
-        <f>S45+W45+X45</f>
+        <f>O45+Q45+S45+U45+W45+X45</f>
       </c>
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B46" s="3"/>
+      <c r="O46" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="2">
+        <v>0</v>
+      </c>
       <c r="S46" s="2">
         <v>0</v>
       </c>
+      <c r="U46" s="2">
+        <v>0</v>
+      </c>
       <c r="W46" s="2">
         <v>0</v>
       </c>
@@ -730,14 +883,23 @@
         <v>0</v>
       </c>
       <c r="Y46" s="2">
-        <f>S46+W46+X46</f>
+        <f>O46+Q46+S46+U46+W46+X46</f>
       </c>
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B47" s="3"/>
+      <c r="O47" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="2">
+        <v>0</v>
+      </c>
       <c r="S47" s="2">
         <v>0</v>
       </c>
+      <c r="U47" s="2">
+        <v>0</v>
+      </c>
       <c r="W47" s="2">
         <v>0</v>
       </c>
@@ -745,14 +907,23 @@
         <v>0</v>
       </c>
       <c r="Y47" s="2">
-        <f>S47+W47+X47</f>
+        <f>O47+Q47+S47+U47+W47+X47</f>
       </c>
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B48" s="3"/>
+      <c r="O48" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="2">
+        <v>0</v>
+      </c>
       <c r="S48" s="2">
         <v>0</v>
       </c>
+      <c r="U48" s="2">
+        <v>0</v>
+      </c>
       <c r="W48" s="2">
         <v>0</v>
       </c>
@@ -760,14 +931,23 @@
         <v>0</v>
       </c>
       <c r="Y48" s="2">
-        <f>S48+W48+X48</f>
+        <f>O48+Q48+S48+U48+W48+X48</f>
       </c>
     </row>
     <row r="49" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B49" s="3"/>
+      <c r="O49" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="2">
+        <v>0</v>
+      </c>
       <c r="S49" s="2">
         <v>0</v>
       </c>
+      <c r="U49" s="2">
+        <v>0</v>
+      </c>
       <c r="W49" s="2">
         <v>0</v>
       </c>
@@ -775,14 +955,23 @@
         <v>0</v>
       </c>
       <c r="Y49" s="2">
-        <f>S49+W49+X49</f>
+        <f>O49+Q49+S49+U49+W49+X49</f>
       </c>
     </row>
     <row r="50" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B50" s="3"/>
+      <c r="O50" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="2">
+        <v>0</v>
+      </c>
       <c r="S50" s="2">
         <v>0</v>
       </c>
+      <c r="U50" s="2">
+        <v>0</v>
+      </c>
       <c r="W50" s="2">
         <v>0</v>
       </c>
@@ -790,14 +979,23 @@
         <v>0</v>
       </c>
       <c r="Y50" s="2">
-        <f>S50+W50+X50</f>
+        <f>O50+Q50+S50+U50+W50+X50</f>
       </c>
     </row>
     <row r="51" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B51" s="3"/>
+      <c r="O51" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="2">
+        <v>0</v>
+      </c>
       <c r="S51" s="2">
         <v>0</v>
       </c>
+      <c r="U51" s="2">
+        <v>0</v>
+      </c>
       <c r="W51" s="2">
         <v>0</v>
       </c>
@@ -805,14 +1003,23 @@
         <v>0</v>
       </c>
       <c r="Y51" s="2">
-        <f>S51+W51+X51</f>
+        <f>O51+Q51+S51+U51+W51+X51</f>
       </c>
     </row>
     <row r="52" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B52" s="3"/>
+      <c r="O52" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="2">
+        <v>0</v>
+      </c>
       <c r="S52" s="2">
         <v>0</v>
       </c>
+      <c r="U52" s="2">
+        <v>0</v>
+      </c>
       <c r="W52" s="2">
         <v>0</v>
       </c>
@@ -820,14 +1027,23 @@
         <v>0</v>
       </c>
       <c r="Y52" s="2">
-        <f>S52+W52+X52</f>
+        <f>O52+Q52+S52+U52+W52+X52</f>
       </c>
     </row>
     <row r="53" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B53" s="3"/>
+      <c r="O53" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="2">
+        <v>0</v>
+      </c>
       <c r="S53" s="2">
         <v>0</v>
       </c>
+      <c r="U53" s="2">
+        <v>0</v>
+      </c>
       <c r="W53" s="2">
         <v>0</v>
       </c>
@@ -835,14 +1051,23 @@
         <v>0</v>
       </c>
       <c r="Y53" s="2">
-        <f>S53+W53+X53</f>
+        <f>O53+Q53+S53+U53+W53+X53</f>
       </c>
     </row>
     <row r="54" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B54" s="3"/>
+      <c r="O54" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="2">
+        <v>0</v>
+      </c>
       <c r="S54" s="2">
         <v>0</v>
       </c>
+      <c r="U54" s="2">
+        <v>0</v>
+      </c>
       <c r="W54" s="2">
         <v>0</v>
       </c>
@@ -850,14 +1075,23 @@
         <v>0</v>
       </c>
       <c r="Y54" s="2">
-        <f>S54+W54+X54</f>
+        <f>O54+Q54+S54+U54+W54+X54</f>
       </c>
     </row>
     <row r="55" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B55" s="3"/>
+      <c r="O55" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="2">
+        <v>0</v>
+      </c>
       <c r="S55" s="2">
         <v>0</v>
       </c>
+      <c r="U55" s="2">
+        <v>0</v>
+      </c>
       <c r="W55" s="2">
         <v>0</v>
       </c>
@@ -865,14 +1099,23 @@
         <v>0</v>
       </c>
       <c r="Y55" s="2">
-        <f>S55+W55+X55</f>
+        <f>O55+Q55+S55+U55+W55+X55</f>
       </c>
     </row>
     <row r="56" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B56" s="3"/>
+      <c r="O56" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="2">
+        <v>0</v>
+      </c>
       <c r="S56" s="2">
         <v>0</v>
       </c>
+      <c r="U56" s="2">
+        <v>0</v>
+      </c>
       <c r="W56" s="2">
         <v>0</v>
       </c>
@@ -880,14 +1123,23 @@
         <v>0</v>
       </c>
       <c r="Y56" s="2">
-        <f>S56+W56+X56</f>
+        <f>O56+Q56+S56+U56+W56+X56</f>
       </c>
     </row>
     <row r="57" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B57" s="3"/>
+      <c r="O57" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="2">
+        <v>0</v>
+      </c>
       <c r="S57" s="2">
         <v>0</v>
       </c>
+      <c r="U57" s="2">
+        <v>0</v>
+      </c>
       <c r="W57" s="2">
         <v>0</v>
       </c>
@@ -895,14 +1147,23 @@
         <v>0</v>
       </c>
       <c r="Y57" s="2">
-        <f>S57+W57+X57</f>
+        <f>O57+Q57+S57+U57+W57+X57</f>
       </c>
     </row>
     <row r="58" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B58" s="3"/>
+      <c r="O58" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="2">
+        <v>0</v>
+      </c>
       <c r="S58" s="2">
         <v>0</v>
       </c>
+      <c r="U58" s="2">
+        <v>0</v>
+      </c>
       <c r="W58" s="2">
         <v>0</v>
       </c>
@@ -910,14 +1171,23 @@
         <v>0</v>
       </c>
       <c r="Y58" s="2">
-        <f>S58+W58+X58</f>
+        <f>O58+Q58+S58+U58+W58+X58</f>
       </c>
     </row>
     <row r="59" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B59" s="3"/>
+      <c r="O59" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="2">
+        <v>0</v>
+      </c>
       <c r="S59" s="2">
         <v>0</v>
       </c>
+      <c r="U59" s="2">
+        <v>0</v>
+      </c>
       <c r="W59" s="2">
         <v>0</v>
       </c>
@@ -925,14 +1195,23 @@
         <v>0</v>
       </c>
       <c r="Y59" s="2">
-        <f>S59+W59+X59</f>
+        <f>O59+Q59+S59+U59+W59+X59</f>
       </c>
     </row>
     <row r="60" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B60" s="3"/>
+      <c r="O60" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="2">
+        <v>0</v>
+      </c>
       <c r="S60" s="2">
         <v>0</v>
       </c>
+      <c r="U60" s="2">
+        <v>0</v>
+      </c>
       <c r="W60" s="2">
         <v>0</v>
       </c>
@@ -940,14 +1219,23 @@
         <v>0</v>
       </c>
       <c r="Y60" s="2">
-        <f>S60+W60+X60</f>
+        <f>O60+Q60+S60+U60+W60+X60</f>
       </c>
     </row>
     <row r="61" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B61" s="3"/>
+      <c r="O61" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="2">
+        <v>0</v>
+      </c>
       <c r="S61" s="2">
         <v>0</v>
       </c>
+      <c r="U61" s="2">
+        <v>0</v>
+      </c>
       <c r="W61" s="2">
         <v>0</v>
       </c>
@@ -955,14 +1243,23 @@
         <v>0</v>
       </c>
       <c r="Y61" s="2">
-        <f>S61+W61+X61</f>
+        <f>O61+Q61+S61+U61+W61+X61</f>
       </c>
     </row>
     <row r="62" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B62" s="3"/>
+      <c r="O62" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="2">
+        <v>0</v>
+      </c>
       <c r="S62" s="2">
         <v>0</v>
       </c>
+      <c r="U62" s="2">
+        <v>0</v>
+      </c>
       <c r="W62" s="2">
         <v>0</v>
       </c>
@@ -970,14 +1267,23 @@
         <v>0</v>
       </c>
       <c r="Y62" s="2">
-        <f>S62+W62+X62</f>
+        <f>O62+Q62+S62+U62+W62+X62</f>
       </c>
     </row>
     <row r="63" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B63" s="3"/>
+      <c r="O63" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q63" s="2">
+        <v>0</v>
+      </c>
       <c r="S63" s="2">
         <v>0</v>
       </c>
+      <c r="U63" s="2">
+        <v>0</v>
+      </c>
       <c r="W63" s="2">
         <v>0</v>
       </c>
@@ -985,14 +1291,23 @@
         <v>0</v>
       </c>
       <c r="Y63" s="2">
-        <f>S63+W63+X63</f>
+        <f>O63+Q63+S63+U63+W63+X63</f>
       </c>
     </row>
     <row r="64" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B64" s="3"/>
+      <c r="O64" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q64" s="2">
+        <v>0</v>
+      </c>
       <c r="S64" s="2">
         <v>0</v>
       </c>
+      <c r="U64" s="2">
+        <v>0</v>
+      </c>
       <c r="W64" s="2">
         <v>0</v>
       </c>
@@ -1000,14 +1315,23 @@
         <v>0</v>
       </c>
       <c r="Y64" s="2">
-        <f>S64+W64+X64</f>
+        <f>O64+Q64+S64+U64+W64+X64</f>
       </c>
     </row>
     <row r="65" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B65" s="3"/>
+      <c r="O65" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q65" s="2">
+        <v>0</v>
+      </c>
       <c r="S65" s="2">
         <v>0</v>
       </c>
+      <c r="U65" s="2">
+        <v>0</v>
+      </c>
       <c r="W65" s="2">
         <v>0</v>
       </c>
@@ -1015,14 +1339,23 @@
         <v>0</v>
       </c>
       <c r="Y65" s="2">
-        <f>S65+W65+X65</f>
+        <f>O65+Q65+S65+U65+W65+X65</f>
       </c>
     </row>
     <row r="66" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B66" s="3"/>
+      <c r="O66" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q66" s="2">
+        <v>0</v>
+      </c>
       <c r="S66" s="2">
         <v>0</v>
       </c>
+      <c r="U66" s="2">
+        <v>0</v>
+      </c>
       <c r="W66" s="2">
         <v>0</v>
       </c>
@@ -1030,14 +1363,23 @@
         <v>0</v>
       </c>
       <c r="Y66" s="2">
-        <f>S66+W66+X66</f>
+        <f>O66+Q66+S66+U66+W66+X66</f>
       </c>
     </row>
     <row r="67" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B67" s="3"/>
+      <c r="O67" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="2">
+        <v>0</v>
+      </c>
       <c r="S67" s="2">
         <v>0</v>
       </c>
+      <c r="U67" s="2">
+        <v>0</v>
+      </c>
       <c r="W67" s="2">
         <v>0</v>
       </c>
@@ -1045,14 +1387,23 @@
         <v>0</v>
       </c>
       <c r="Y67" s="2">
-        <f>S67+W67+X67</f>
+        <f>O67+Q67+S67+U67+W67+X67</f>
       </c>
     </row>
     <row r="68" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B68" s="3"/>
+      <c r="O68" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="2">
+        <v>0</v>
+      </c>
       <c r="S68" s="2">
         <v>0</v>
       </c>
+      <c r="U68" s="2">
+        <v>0</v>
+      </c>
       <c r="W68" s="2">
         <v>0</v>
       </c>
@@ -1060,14 +1411,23 @@
         <v>0</v>
       </c>
       <c r="Y68" s="2">
-        <f>S68+W68+X68</f>
+        <f>O68+Q68+S68+U68+W68+X68</f>
       </c>
     </row>
     <row r="69" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B69" s="3"/>
+      <c r="O69" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="2">
+        <v>0</v>
+      </c>
       <c r="S69" s="2">
         <v>0</v>
       </c>
+      <c r="U69" s="2">
+        <v>0</v>
+      </c>
       <c r="W69" s="2">
         <v>0</v>
       </c>
@@ -1075,14 +1435,23 @@
         <v>0</v>
       </c>
       <c r="Y69" s="2">
-        <f>S69+W69+X69</f>
+        <f>O69+Q69+S69+U69+W69+X69</f>
       </c>
     </row>
     <row r="70" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B70" s="3"/>
+      <c r="O70" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="2">
+        <v>0</v>
+      </c>
       <c r="S70" s="2">
         <v>0</v>
       </c>
+      <c r="U70" s="2">
+        <v>0</v>
+      </c>
       <c r="W70" s="2">
         <v>0</v>
       </c>
@@ -1090,14 +1459,23 @@
         <v>0</v>
       </c>
       <c r="Y70" s="2">
-        <f>S70+W70+X70</f>
+        <f>O70+Q70+S70+U70+W70+X70</f>
       </c>
     </row>
     <row r="71" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B71" s="3"/>
+      <c r="O71" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="2">
+        <v>0</v>
+      </c>
       <c r="S71" s="2">
         <v>0</v>
       </c>
+      <c r="U71" s="2">
+        <v>0</v>
+      </c>
       <c r="W71" s="2">
         <v>0</v>
       </c>
@@ -1105,14 +1483,23 @@
         <v>0</v>
       </c>
       <c r="Y71" s="2">
-        <f>S71+W71+X71</f>
+        <f>O71+Q71+S71+U71+W71+X71</f>
       </c>
     </row>
     <row r="72" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B72" s="3"/>
+      <c r="O72" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="2">
+        <v>0</v>
+      </c>
       <c r="S72" s="2">
         <v>0</v>
       </c>
+      <c r="U72" s="2">
+        <v>0</v>
+      </c>
       <c r="W72" s="2">
         <v>0</v>
       </c>
@@ -1120,14 +1507,23 @@
         <v>0</v>
       </c>
       <c r="Y72" s="2">
-        <f>S72+W72+X72</f>
+        <f>O72+Q72+S72+U72+W72+X72</f>
       </c>
     </row>
     <row r="73" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B73" s="3"/>
+      <c r="O73" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q73" s="2">
+        <v>0</v>
+      </c>
       <c r="S73" s="2">
         <v>0</v>
       </c>
+      <c r="U73" s="2">
+        <v>0</v>
+      </c>
       <c r="W73" s="2">
         <v>0</v>
       </c>
@@ -1135,14 +1531,23 @@
         <v>0</v>
       </c>
       <c r="Y73" s="2">
-        <f>S73+W73+X73</f>
+        <f>O73+Q73+S73+U73+W73+X73</f>
       </c>
     </row>
     <row r="74" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B74" s="3"/>
+      <c r="O74" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q74" s="2">
+        <v>0</v>
+      </c>
       <c r="S74" s="2">
         <v>0</v>
       </c>
+      <c r="U74" s="2">
+        <v>0</v>
+      </c>
       <c r="W74" s="2">
         <v>0</v>
       </c>
@@ -1150,14 +1555,23 @@
         <v>0</v>
       </c>
       <c r="Y74" s="2">
-        <f>S74+W74+X74</f>
+        <f>O74+Q74+S74+U74+W74+X74</f>
       </c>
     </row>
     <row r="75" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B75" s="3"/>
+      <c r="O75" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q75" s="2">
+        <v>0</v>
+      </c>
       <c r="S75" s="2">
         <v>0</v>
       </c>
+      <c r="U75" s="2">
+        <v>0</v>
+      </c>
       <c r="W75" s="2">
         <v>0</v>
       </c>
@@ -1165,14 +1579,23 @@
         <v>0</v>
       </c>
       <c r="Y75" s="2">
-        <f>S75+W75+X75</f>
+        <f>O75+Q75+S75+U75+W75+X75</f>
       </c>
     </row>
     <row r="76" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B76" s="3"/>
+      <c r="O76" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="2">
+        <v>0</v>
+      </c>
       <c r="S76" s="2">
         <v>0</v>
       </c>
+      <c r="U76" s="2">
+        <v>0</v>
+      </c>
       <c r="W76" s="2">
         <v>0</v>
       </c>
@@ -1180,14 +1603,23 @@
         <v>0</v>
       </c>
       <c r="Y76" s="2">
-        <f>S76+W76+X76</f>
+        <f>O76+Q76+S76+U76+W76+X76</f>
       </c>
     </row>
     <row r="77" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B77" s="3"/>
+      <c r="O77" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="2">
+        <v>0</v>
+      </c>
       <c r="S77" s="2">
         <v>0</v>
       </c>
+      <c r="U77" s="2">
+        <v>0</v>
+      </c>
       <c r="W77" s="2">
         <v>0</v>
       </c>
@@ -1195,14 +1627,23 @@
         <v>0</v>
       </c>
       <c r="Y77" s="2">
-        <f>S77+W77+X77</f>
+        <f>O77+Q77+S77+U77+W77+X77</f>
       </c>
     </row>
     <row r="78" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B78" s="3"/>
+      <c r="O78" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="2">
+        <v>0</v>
+      </c>
       <c r="S78" s="2">
         <v>0</v>
       </c>
+      <c r="U78" s="2">
+        <v>0</v>
+      </c>
       <c r="W78" s="2">
         <v>0</v>
       </c>
@@ -1210,14 +1651,23 @@
         <v>0</v>
       </c>
       <c r="Y78" s="2">
-        <f>S78+W78+X78</f>
+        <f>O78+Q78+S78+U78+W78+X78</f>
       </c>
     </row>
     <row r="79" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B79" s="3"/>
+      <c r="O79" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="2">
+        <v>0</v>
+      </c>
       <c r="S79" s="2">
         <v>0</v>
       </c>
+      <c r="U79" s="2">
+        <v>0</v>
+      </c>
       <c r="W79" s="2">
         <v>0</v>
       </c>
@@ -1225,14 +1675,23 @@
         <v>0</v>
       </c>
       <c r="Y79" s="2">
-        <f>S79+W79+X79</f>
+        <f>O79+Q79+S79+U79+W79+X79</f>
       </c>
     </row>
     <row r="80" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B80" s="3"/>
+      <c r="O80" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="2">
+        <v>0</v>
+      </c>
       <c r="S80" s="2">
         <v>0</v>
       </c>
+      <c r="U80" s="2">
+        <v>0</v>
+      </c>
       <c r="W80" s="2">
         <v>0</v>
       </c>
@@ -1240,14 +1699,23 @@
         <v>0</v>
       </c>
       <c r="Y80" s="2">
-        <f>S80+W80+X80</f>
+        <f>O80+Q80+S80+U80+W80+X80</f>
       </c>
     </row>
     <row r="81" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B81" s="3"/>
+      <c r="O81" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q81" s="2">
+        <v>0</v>
+      </c>
       <c r="S81" s="2">
         <v>0</v>
       </c>
+      <c r="U81" s="2">
+        <v>0</v>
+      </c>
       <c r="W81" s="2">
         <v>0</v>
       </c>
@@ -1255,14 +1723,23 @@
         <v>0</v>
       </c>
       <c r="Y81" s="2">
-        <f>S81+W81+X81</f>
+        <f>O81+Q81+S81+U81+W81+X81</f>
       </c>
     </row>
     <row r="82" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B82" s="3"/>
+      <c r="O82" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q82" s="2">
+        <v>0</v>
+      </c>
       <c r="S82" s="2">
         <v>0</v>
       </c>
+      <c r="U82" s="2">
+        <v>0</v>
+      </c>
       <c r="W82" s="2">
         <v>0</v>
       </c>
@@ -1270,14 +1747,23 @@
         <v>0</v>
       </c>
       <c r="Y82" s="2">
-        <f>S82+W82+X82</f>
+        <f>O82+Q82+S82+U82+W82+X82</f>
       </c>
     </row>
     <row r="83" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B83" s="3"/>
+      <c r="O83" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q83" s="2">
+        <v>0</v>
+      </c>
       <c r="S83" s="2">
         <v>0</v>
       </c>
+      <c r="U83" s="2">
+        <v>0</v>
+      </c>
       <c r="W83" s="2">
         <v>0</v>
       </c>
@@ -1285,14 +1771,23 @@
         <v>0</v>
       </c>
       <c r="Y83" s="2">
-        <f>S83+W83+X83</f>
+        <f>O83+Q83+S83+U83+W83+X83</f>
       </c>
     </row>
     <row r="84" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B84" s="3"/>
+      <c r="O84" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q84" s="2">
+        <v>0</v>
+      </c>
       <c r="S84" s="2">
         <v>0</v>
       </c>
+      <c r="U84" s="2">
+        <v>0</v>
+      </c>
       <c r="W84" s="2">
         <v>0</v>
       </c>
@@ -1300,14 +1795,23 @@
         <v>0</v>
       </c>
       <c r="Y84" s="2">
-        <f>S84+W84+X84</f>
+        <f>O84+Q84+S84+U84+W84+X84</f>
       </c>
     </row>
     <row r="85" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B85" s="3"/>
+      <c r="O85" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q85" s="2">
+        <v>0</v>
+      </c>
       <c r="S85" s="2">
         <v>0</v>
       </c>
+      <c r="U85" s="2">
+        <v>0</v>
+      </c>
       <c r="W85" s="2">
         <v>0</v>
       </c>
@@ -1315,14 +1819,23 @@
         <v>0</v>
       </c>
       <c r="Y85" s="2">
-        <f>S85+W85+X85</f>
+        <f>O85+Q85+S85+U85+W85+X85</f>
       </c>
     </row>
     <row r="86" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B86" s="3"/>
+      <c r="O86" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="2">
+        <v>0</v>
+      </c>
       <c r="S86" s="2">
         <v>0</v>
       </c>
+      <c r="U86" s="2">
+        <v>0</v>
+      </c>
       <c r="W86" s="2">
         <v>0</v>
       </c>
@@ -1330,14 +1843,23 @@
         <v>0</v>
       </c>
       <c r="Y86" s="2">
-        <f>S86+W86+X86</f>
+        <f>O86+Q86+S86+U86+W86+X86</f>
       </c>
     </row>
     <row r="87" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B87" s="3"/>
+      <c r="O87" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q87" s="2">
+        <v>0</v>
+      </c>
       <c r="S87" s="2">
         <v>0</v>
       </c>
+      <c r="U87" s="2">
+        <v>0</v>
+      </c>
       <c r="W87" s="2">
         <v>0</v>
       </c>
@@ -1345,14 +1867,23 @@
         <v>0</v>
       </c>
       <c r="Y87" s="2">
-        <f>S87+W87+X87</f>
+        <f>O87+Q87+S87+U87+W87+X87</f>
       </c>
     </row>
     <row r="88" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B88" s="3"/>
+      <c r="O88" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="2">
+        <v>0</v>
+      </c>
       <c r="S88" s="2">
         <v>0</v>
       </c>
+      <c r="U88" s="2">
+        <v>0</v>
+      </c>
       <c r="W88" s="2">
         <v>0</v>
       </c>
@@ -1360,14 +1891,23 @@
         <v>0</v>
       </c>
       <c r="Y88" s="2">
-        <f>S88+W88+X88</f>
+        <f>O88+Q88+S88+U88+W88+X88</f>
       </c>
     </row>
     <row r="89" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B89" s="3"/>
+      <c r="O89" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q89" s="2">
+        <v>0</v>
+      </c>
       <c r="S89" s="2">
         <v>0</v>
       </c>
+      <c r="U89" s="2">
+        <v>0</v>
+      </c>
       <c r="W89" s="2">
         <v>0</v>
       </c>
@@ -1375,14 +1915,23 @@
         <v>0</v>
       </c>
       <c r="Y89" s="2">
-        <f>S89+W89+X89</f>
+        <f>O89+Q89+S89+U89+W89+X89</f>
       </c>
     </row>
     <row r="90" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B90" s="3"/>
+      <c r="O90" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="2">
+        <v>0</v>
+      </c>
       <c r="S90" s="2">
         <v>0</v>
       </c>
+      <c r="U90" s="2">
+        <v>0</v>
+      </c>
       <c r="W90" s="2">
         <v>0</v>
       </c>
@@ -1390,14 +1939,23 @@
         <v>0</v>
       </c>
       <c r="Y90" s="2">
-        <f>S90+W90+X90</f>
+        <f>O90+Q90+S90+U90+W90+X90</f>
       </c>
     </row>
     <row r="91" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B91" s="3"/>
+      <c r="O91" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q91" s="2">
+        <v>0</v>
+      </c>
       <c r="S91" s="2">
         <v>0</v>
       </c>
+      <c r="U91" s="2">
+        <v>0</v>
+      </c>
       <c r="W91" s="2">
         <v>0</v>
       </c>
@@ -1405,14 +1963,23 @@
         <v>0</v>
       </c>
       <c r="Y91" s="2">
-        <f>S91+W91+X91</f>
+        <f>O91+Q91+S91+U91+W91+X91</f>
       </c>
     </row>
     <row r="92" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B92" s="3"/>
+      <c r="O92" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q92" s="2">
+        <v>0</v>
+      </c>
       <c r="S92" s="2">
         <v>0</v>
       </c>
+      <c r="U92" s="2">
+        <v>0</v>
+      </c>
       <c r="W92" s="2">
         <v>0</v>
       </c>
@@ -1420,14 +1987,23 @@
         <v>0</v>
       </c>
       <c r="Y92" s="2">
-        <f>S92+W92+X92</f>
+        <f>O92+Q92+S92+U92+W92+X92</f>
       </c>
     </row>
     <row r="93" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B93" s="3"/>
+      <c r="O93" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q93" s="2">
+        <v>0</v>
+      </c>
       <c r="S93" s="2">
         <v>0</v>
       </c>
+      <c r="U93" s="2">
+        <v>0</v>
+      </c>
       <c r="W93" s="2">
         <v>0</v>
       </c>
@@ -1435,14 +2011,23 @@
         <v>0</v>
       </c>
       <c r="Y93" s="2">
-        <f>S93+W93+X93</f>
+        <f>O93+Q93+S93+U93+W93+X93</f>
       </c>
     </row>
     <row r="94" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B94" s="3"/>
+      <c r="O94" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q94" s="2">
+        <v>0</v>
+      </c>
       <c r="S94" s="2">
         <v>0</v>
       </c>
+      <c r="U94" s="2">
+        <v>0</v>
+      </c>
       <c r="W94" s="2">
         <v>0</v>
       </c>
@@ -1450,14 +2035,23 @@
         <v>0</v>
       </c>
       <c r="Y94" s="2">
-        <f>S94+W94+X94</f>
+        <f>O94+Q94+S94+U94+W94+X94</f>
       </c>
     </row>
     <row r="95" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B95" s="3"/>
+      <c r="O95" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q95" s="2">
+        <v>0</v>
+      </c>
       <c r="S95" s="2">
         <v>0</v>
       </c>
+      <c r="U95" s="2">
+        <v>0</v>
+      </c>
       <c r="W95" s="2">
         <v>0</v>
       </c>
@@ -1465,14 +2059,23 @@
         <v>0</v>
       </c>
       <c r="Y95" s="2">
-        <f>S95+W95+X95</f>
+        <f>O95+Q95+S95+U95+W95+X95</f>
       </c>
     </row>
     <row r="96" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B96" s="3"/>
+      <c r="O96" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q96" s="2">
+        <v>0</v>
+      </c>
       <c r="S96" s="2">
         <v>0</v>
       </c>
+      <c r="U96" s="2">
+        <v>0</v>
+      </c>
       <c r="W96" s="2">
         <v>0</v>
       </c>
@@ -1480,14 +2083,23 @@
         <v>0</v>
       </c>
       <c r="Y96" s="2">
-        <f>S96+W96+X96</f>
+        <f>O96+Q96+S96+U96+W96+X96</f>
       </c>
     </row>
     <row r="97" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B97" s="3"/>
+      <c r="O97" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q97" s="2">
+        <v>0</v>
+      </c>
       <c r="S97" s="2">
         <v>0</v>
       </c>
+      <c r="U97" s="2">
+        <v>0</v>
+      </c>
       <c r="W97" s="2">
         <v>0</v>
       </c>
@@ -1495,14 +2107,23 @@
         <v>0</v>
       </c>
       <c r="Y97" s="2">
-        <f>S97+W97+X97</f>
+        <f>O97+Q97+S97+U97+W97+X97</f>
       </c>
     </row>
     <row r="98" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B98" s="3"/>
+      <c r="O98" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q98" s="2">
+        <v>0</v>
+      </c>
       <c r="S98" s="2">
         <v>0</v>
       </c>
+      <c r="U98" s="2">
+        <v>0</v>
+      </c>
       <c r="W98" s="2">
         <v>0</v>
       </c>
@@ -1510,14 +2131,23 @@
         <v>0</v>
       </c>
       <c r="Y98" s="2">
-        <f>S98+W98+X98</f>
+        <f>O98+Q98+S98+U98+W98+X98</f>
       </c>
     </row>
     <row r="99" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B99" s="3"/>
+      <c r="O99" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q99" s="2">
+        <v>0</v>
+      </c>
       <c r="S99" s="2">
         <v>0</v>
       </c>
+      <c r="U99" s="2">
+        <v>0</v>
+      </c>
       <c r="W99" s="2">
         <v>0</v>
       </c>
@@ -1525,14 +2155,23 @@
         <v>0</v>
       </c>
       <c r="Y99" s="2">
-        <f>S99+W99+X99</f>
+        <f>O99+Q99+S99+U99+W99+X99</f>
       </c>
     </row>
     <row r="100" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B100" s="3"/>
+      <c r="O100" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q100" s="2">
+        <v>0</v>
+      </c>
       <c r="S100" s="2">
         <v>0</v>
       </c>
+      <c r="U100" s="2">
+        <v>0</v>
+      </c>
       <c r="W100" s="2">
         <v>0</v>
       </c>
@@ -1540,15 +2179,24 @@
         <v>0</v>
       </c>
       <c r="Y100" s="2">
-        <f>S100+W100+X100</f>
+        <f>O100+Q100+S100+U100+W100+X100</f>
       </c>
     </row>
     <row r="101" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B101" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="O101" s="4">
+        <f>SUM(O32:O100)</f>
+      </c>
+      <c r="Q101" s="4">
+        <f>SUM(Q32:Q100)</f>
       </c>
       <c r="S101" s="4">
         <f>SUM(S32:S100)</f>
+      </c>
+      <c r="U101" s="4">
+        <f>SUM(U32:U100)</f>
       </c>
       <c r="W101" s="4">
         <f>SUM(W32:W100)</f>

</xml_diff>